<commit_message>
Add paper annotation files and update pepline outputs
Add paper/VEA_Annot_table.csv, VEA_Annot_table.xlsx, VEA_new_annot_example.xlsx and an annot_table.py helper (plus paper/.DS_Store). Rename/remove several Office temporary (~$...) files and update repository .DS_Store entries. Also update pepline: modify pepline_test.ipynb, pepline/.DS_Store and replace pepline/result/deconv_result.xlsx with a new version. These changes add the annotation data and script for the paper and refresh pipeline results and metadata.
</commit_message>
<xml_diff>
--- a/pepline/result/deconv_result.xlsx
+++ b/pepline/result/deconv_result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinmbp/Desktop/2D_spec_dict/pepline/result/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF6FD86B-A4CB-2649-B9FE-0FED048327DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FE9AD6-4972-8F47-856D-258D8F48BDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5260" yWindow="4660" windowWidth="44780" windowHeight="20980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5260" yWindow="4660" windowWidth="44780" windowHeight="20980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3+_nondeconv" sheetId="3" r:id="rId1"/>
@@ -3205,7 +3205,7 @@
       </c>
     </row>
     <row r="34" spans="1:17">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>117</v>
       </c>
       <c r="E34">
@@ -3237,7 +3237,7 @@
       </c>
     </row>
     <row r="35" spans="1:17">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>118</v>
       </c>
       <c r="E35">

</xml_diff>